<commit_message>
Replace bot FAQ with indexed Article source; simplify Knowledge Base link scan
- Chatbot Knowledge: FAQ (instant Q&A) replaced by Article, a proper
  trainable source (title + content) sharing the same indexed/indexing/
  queued/failed lifecycle as documents and URLs, with its own table,
  retrain/enable-disable/delete actions, and in-place editing
- Chat composer's knowledge-base quick replies now rank articles and
  exclude any that aren't indexed yet, not just disabled ones
- Add Document dialog: dropped the signed-in audience picker (matches
  the earlier change to Add URL) — new documents are always public
- Knowledge Base "Add website link" dialog: replaced scan depth/max
  pages selects with the same single-page/multiple-pages choice used
  for bot training URLs
- Synced v1 docs (AI-07, FEAT-009/020, FE-17, Requirements Overview) to
  the FAQ -> Article terminology and regenerated all deliverables

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/v1/Mercury_V1_Feature_Listing.xlsx
+++ b/docs/v1/Mercury_V1_Feature_Listing.xlsx
@@ -1006,13 +1006,13 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>In-chat panel that searches Internal Knowledge and suggests trained FAQs relevant to the conversation's matched bot intent.</t>
+          <t>In-chat panel that searches Internal Knowledge and suggests trained articles relevant to the conversation's matched bot intent.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>- Ask Knowledge search panel
-- Suggested-reply dialog ranking FAQs by matched intent
+- Quick-reply menu ranking trained articles by matched intent
 - Editable draft only (never auto-sent)</t>
         </is>
       </c>
@@ -1448,7 +1448,7 @@
         <is>
           <t>- Articles tab: create/edit, category, groups, pin, review status (current/due/stale/draft)
 - Documents tab: upload/add internal document
-- Links tab: add internal reference link</t>
+- Links tab: add an internal reference link as a single page or a multi-page site scan</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1556,12 +1556,12 @@
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>- Add source document
-- Add source URL with crawl depth
+- Add source URL as a single page or a multi-page site scan (admin-configurable scan depth/page-limit deferred to V2 — see AI-13/BE-15)
 - Enable / disable a source ('use for answers')
 - Retrain a source
 - Delete a source
 - Training status: indexed/indexing/queued/failed + failure reason
-- Public vs. signed-in audience setting</t>
+- Audience badge (public/signed-in) shown per source; audience is no longer admin-settable when adding a source in V1 — every new document or URL source is public by default</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1603,18 +1603,18 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Bot FAQ Management</t>
+          <t>Bot Article Management</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Structured FAQs the bot can answer from directly, each tagged with the intents it matches.</t>
+          <t>Structured articles (title + content) the bot can answer from directly, each tagged with the intents it matches. Same indexing lifecycle as documents/URLs (status, chunks, retrain) rather than an instant, unindexed Q&amp;A pair.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>- Add / edit FAQ (category, question, answer)
-- Tag FAQ with matched bot intents
+          <t>- Add / edit article (category, title, content)
+- Tag article with matched bot intents
 - Feeds Chat's suggested-reply ranking</t>
         </is>
       </c>

</xml_diff>